<commit_message>
Se agregraron las validaciones necesarias para que el sistema no permita registros hasta que se haya cargado el presupuesto y los saldos iniciales
</commit_message>
<xml_diff>
--- a/public/PresupuestoInicial/Poliza Inicial v2.xlsx
+++ b/public/PresupuestoInicial/Poliza Inicial v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\SAC-IPE\public\PresupuestoInicial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C446ADD-711D-4A31-B171-39728BC7A075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91BFEA5-1E9A-4827-9324-1531821E4283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="840" xr2:uid="{1ABF5C7F-72DD-4BD5-835F-CAF0BF8EAFC5}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="840" xr2:uid="{1ABF5C7F-72DD-4BD5-835F-CAF0BF8EAFC5}"/>
   </bookViews>
   <sheets>
     <sheet name="POLIZA PRUEBA TECNOLOGIAS" sheetId="17" r:id="rId1"/>
@@ -1336,7 +1336,7 @@
         <v>85</v>
       </c>
       <c r="C3" s="3">
-        <v>5030912.280000153</v>
+        <v>5030912.28</v>
       </c>
       <c r="E3" t="s">
         <v>139</v>
@@ -1420,7 +1420,7 @@
         <v>101</v>
       </c>
       <c r="C9" s="3">
-        <v>4789717.675999999</v>
+        <v>4789717.67</v>
       </c>
       <c r="E9" t="s">
         <v>139</v>
@@ -1462,7 +1462,7 @@
         <v>8</v>
       </c>
       <c r="C12" s="3">
-        <v>7259171.2219999693</v>
+        <v>7259171.2199999997</v>
       </c>
       <c r="E12" t="s">
         <v>139</v>
@@ -1602,7 +1602,7 @@
         <v>145</v>
       </c>
       <c r="C22" s="4">
-        <v>12067744.582</v>
+        <v>12067744.58</v>
       </c>
       <c r="E22" t="s">
         <v>139</v>
@@ -1742,7 +1742,7 @@
         <v>136</v>
       </c>
       <c r="C32" s="4">
-        <v>265818246.87500003</v>
+        <v>265818246.87</v>
       </c>
       <c r="E32" t="s">
         <v>139</v>
@@ -1756,7 +1756,7 @@
         <v>20</v>
       </c>
       <c r="C33" s="5">
-        <v>615911.88406816381</v>
+        <v>615911.88</v>
       </c>
       <c r="E33" t="s">
         <v>139</v>
@@ -1770,7 +1770,7 @@
         <v>21</v>
       </c>
       <c r="C34" s="5">
-        <v>2556343.3448425638</v>
+        <v>2556343.34</v>
       </c>
       <c r="E34" t="s">
         <v>139</v>
@@ -1784,7 +1784,7 @@
         <v>23</v>
       </c>
       <c r="C35" s="5">
-        <v>34801.649000000012</v>
+        <v>34801.64</v>
       </c>
       <c r="E35" t="s">
         <v>139</v>
@@ -1798,7 +1798,7 @@
         <v>25</v>
       </c>
       <c r="C36" s="5">
-        <v>1059043.9312546314</v>
+        <v>1059043.93</v>
       </c>
       <c r="E36" t="s">
         <v>139</v>
@@ -1826,7 +1826,7 @@
         <v>27</v>
       </c>
       <c r="C38" s="5">
-        <v>98906.146800000002</v>
+        <v>98906.14</v>
       </c>
       <c r="E38" t="s">
         <v>139</v>
@@ -1840,7 +1840,7 @@
         <v>28</v>
       </c>
       <c r="C39" s="5">
-        <v>1211367.5394236788</v>
+        <v>1211367.53</v>
       </c>
       <c r="E39" t="s">
         <v>139</v>
@@ -1854,7 +1854,7 @@
         <v>29</v>
       </c>
       <c r="C40" s="5">
-        <v>1027144.490864502</v>
+        <v>1027144.49</v>
       </c>
       <c r="E40" t="s">
         <v>139</v>
@@ -1868,7 +1868,7 @@
         <v>30</v>
       </c>
       <c r="C41" s="5">
-        <v>181504.81520000001</v>
+        <v>181504.81</v>
       </c>
       <c r="E41" t="s">
         <v>139</v>
@@ -1882,7 +1882,7 @@
         <v>31</v>
       </c>
       <c r="C42" s="5">
-        <v>157355.30980000002</v>
+        <v>157355.29999999999</v>
       </c>
       <c r="E42" t="s">
         <v>139</v>
@@ -1896,7 +1896,7 @@
         <v>32</v>
       </c>
       <c r="C43" s="5">
-        <v>50851.812500000029</v>
+        <v>50851.81</v>
       </c>
       <c r="E43" t="s">
         <v>139</v>
@@ -1910,7 +1910,7 @@
         <v>33</v>
       </c>
       <c r="C44" s="5">
-        <v>131106.02059999996</v>
+        <v>131106.01999999999</v>
       </c>
       <c r="E44" t="s">
         <v>139</v>
@@ -1924,7 +1924,7 @@
         <v>34</v>
       </c>
       <c r="C45" s="5">
-        <v>14998.798000000006</v>
+        <v>14998.79</v>
       </c>
       <c r="E45" t="s">
         <v>139</v>
@@ -1938,7 +1938,7 @@
         <v>35</v>
       </c>
       <c r="C46" s="5">
-        <v>53282.281299999988</v>
+        <v>53282.28</v>
       </c>
       <c r="E46" t="s">
         <v>139</v>
@@ -2260,7 +2260,7 @@
         <v>51</v>
       </c>
       <c r="C69" s="11">
-        <v>263872791.57080001</v>
+        <v>263872791.56999999</v>
       </c>
       <c r="E69" t="s">
         <v>140</v>
@@ -2498,7 +2498,7 @@
         <v>130</v>
       </c>
       <c r="D86" s="1">
-        <v>5745663.5460000001</v>
+        <v>5745663.54</v>
       </c>
       <c r="E86" t="s">
         <v>140</v>
@@ -2610,7 +2610,7 @@
         <v>199</v>
       </c>
       <c r="D94" s="1">
-        <v>99402402.335999995</v>
+        <v>99402402.329999998</v>
       </c>
       <c r="E94" t="s">
         <v>140</v>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="C96" s="11"/>
       <c r="D96" s="11">
-        <v>133.26595687866211</v>
+        <v>133.26</v>
       </c>
       <c r="E96" t="s">
         <v>140</v>
@@ -2793,7 +2793,7 @@
         <v>224</v>
       </c>
       <c r="D107" s="1">
-        <v>301481.4852</v>
+        <v>301481.48</v>
       </c>
       <c r="E107" t="s">
         <v>140</v>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="C134" s="11"/>
       <c r="D134" s="11">
-        <v>299459436.56529999</v>
+        <v>299459436.56</v>
       </c>
       <c r="E134" t="s">
         <v>139</v>

</xml_diff>